<commit_message>
add: manager logs user12
</commit_message>
<xml_diff>
--- a/Copy of 0. 131.xlsx
+++ b/Copy of 0. 131.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\.Freelancer\BTTD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC44A6E2-A4D3-48A7-A47C-F6D4F5938D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{978D4152-7514-48A5-B5B4-F2235416E02F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -417,6 +417,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -425,9 +428,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1408,28 +1408,28 @@
       <c r="A6" s="1"/>
     </row>
     <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="27" t="s">
-        <v>0</v>
-      </c>
-      <c r="B7" s="24" t="s">
+      <c r="A7" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="C7" s="24" t="s">
+      <c r="C7" s="25" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="24"/>
-      <c r="E7" s="24" t="s">
+      <c r="D7" s="25"/>
+      <c r="E7" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F7" s="24"/>
-      <c r="G7" s="25" t="s">
+      <c r="F7" s="25"/>
+      <c r="G7" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="H7" s="25"/>
+      <c r="H7" s="26"/>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="27"/>
-      <c r="B8" s="24"/>
+      <c r="A8" s="24"/>
+      <c r="B8" s="25"/>
       <c r="C8" s="5" t="s">
         <v>5</v>
       </c>
@@ -1477,10 +1477,10 @@
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
-      <c r="B10" s="26" t="s">
+      <c r="B10" s="27" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="26"/>
+      <c r="C10" s="27"/>
       <c r="D10" s="12">
         <f>SUBTOTAL(9,D11:D13)</f>
         <v>1457585643</v>
@@ -1586,27 +1586,27 @@
         <v>22</v>
       </c>
       <c r="C14" s="12">
-        <f>SUBTOTAL(9,C15:C15)</f>
+        <f t="shared" ref="C14:H14" si="0">SUBTOTAL(9,C15:C15)</f>
         <v>13000000</v>
       </c>
       <c r="D14" s="12">
-        <f>SUBTOTAL(9,D15:D15)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="E14" s="12">
-        <f>SUBTOTAL(9,E15:E15)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="F14" s="12">
-        <f>SUBTOTAL(9,F15:F15)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
       <c r="G14" s="12">
-        <f>SUBTOTAL(9,G15:G15)</f>
+        <f t="shared" si="0"/>
         <v>13000000</v>
       </c>
       <c r="H14" s="13">
-        <f>SUBTOTAL(9,H15:H15)</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
@@ -1642,27 +1642,27 @@
         <v>25</v>
       </c>
       <c r="C16" s="20">
-        <f>SUBTOTAL(9,C10:C15)</f>
+        <f t="shared" ref="C16:H16" si="1">SUBTOTAL(9,C10:C15)</f>
         <v>13000000</v>
       </c>
       <c r="D16" s="20">
-        <f>SUBTOTAL(9,D10:D15)</f>
+        <f t="shared" si="1"/>
         <v>1457585643</v>
       </c>
       <c r="E16" s="20">
-        <f>SUBTOTAL(9,E10:E15)</f>
+        <f t="shared" si="1"/>
         <v>188802186</v>
       </c>
       <c r="F16" s="20">
-        <f>SUBTOTAL(9,F10:F15)</f>
+        <f t="shared" si="1"/>
         <v>109680000</v>
       </c>
       <c r="G16" s="20">
-        <f>SUBTOTAL(9,G10:G15)</f>
+        <f t="shared" si="1"/>
         <v>13000000</v>
       </c>
       <c r="H16" s="21">
-        <f>SUBTOTAL(9,H10:H15)</f>
+        <f t="shared" si="1"/>
         <v>1378463457</v>
       </c>
     </row>
@@ -1678,12 +1678,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B10:C10"/>
     <mergeCell ref="A7:A8"/>
     <mergeCell ref="B7:B8"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="E7:F7"/>
     <mergeCell ref="G7:H7"/>
-    <mergeCell ref="B10:C10"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.59" bottom="0.59" header="0.5" footer="0.5"/>

</xml_diff>